<commit_message>
n8n board refresh 2026-08-15T17:41:12Z
</commit_message>
<xml_diff>
--- a/app/reports/AMRZ_research.xlsx
+++ b/app/reports/AMRZ_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-15 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.494</v>
+        <v>0.484</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>31.28</v>
+        <v>30.1</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>46.65</v>
+        <v>46.69</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>-0.329</v>
+        <v>-0.355</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.796</v>
+        <v>0.795</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.17</v>
+        <v>0.145</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04644999980926514</v>
+        <v>0.04696000099182129</v>
       </c>
     </row>
     <row r="6">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>6632999936</v>
+        <v>7090999808</v>
       </c>
     </row>
     <row r="33">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>546925665.6806003</v>
+        <v>546925615.592204</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>46.65</v>
+        <v>46.69</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>25514082304</v>
+        <v>25535956992</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>20.92</v>
+        <v>20.94</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.88</v>
+        <v>11.06</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>2.59</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>20591751168</v>
+        <v>20706605056</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>20.916668</v>
+        <v>20.917128</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.314</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>2.215</v>
+        <v>2.221</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>65696841728</v>
+        <v>64632389632</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.020073</v>
+        <v>17.164312</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>10.797</v>
+        <v>10.724</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>2.161</v>
+        <v>2.146</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>48343138304</v>
+        <v>47762354176</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>100.45977</v>
+        <v>100.406975</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>18.956</v>
+        <v>18.762</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.59</v>
+        <v>3.553</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>48509075456</v>
+        <v>48592039936</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>103.176476</v>
+        <v>103.352936</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.095</v>
+        <v>19.04</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.616</v>
+        <v>3.606</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>39559507968</v>
+        <v>39625883648</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>102.171425</v>
+        <v>102.34286</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>16.079</v>
+        <v>16.035</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.045</v>
+        <v>3.037</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>32840095744</v>
+        <v>32911876096</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>35.52534</v>
+        <v>35.579872</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>18.3</v>
+        <v>18.413</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.817</v>
+        <v>5.853</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>2930441472</v>
+        <v>2957174016</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>16.557293</v>
+        <v>16.708334</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.695</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>2.024</v>
+        <v>2.025</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>36171255808</v>
+        <v>36541202432</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>32.956905</v>
+        <v>33.21555</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>17.563</v>
+        <v>17.653</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.065</v>
+        <v>5.09</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-16T17:41:01Z
</commit_message>
<xml_diff>
--- a/app/reports/AMRZ_research.xlsx
+++ b/app/reports/AMRZ_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-15 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-16 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.795</v>
+        <v>0.797</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>

</xml_diff>